<commit_message>
Update q4 schedules and result_tables after test runs
</commit_message>
<xml_diff>
--- a/outputs/result_tables.xlsx
+++ b/outputs/result_tables.xlsx
@@ -841,21 +841,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine1-2</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5600</v>
+        <v>8995</v>
       </c>
       <c r="D11" t="n">
-        <v>23600</v>
+        <v>23395</v>
       </c>
       <c r="E11" t="n">
-        <v>18000</v>
+        <v>14400</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>D2</t>
         </is>
       </c>
     </row>
@@ -865,21 +865,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-5</t>
+          <t>Automated Conveying Arm1-2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5600</v>
+        <v>8995</v>
       </c>
       <c r="D12" t="n">
-        <v>12800</v>
+        <v>18595</v>
       </c>
       <c r="E12" t="n">
-        <v>7200</v>
+        <v>9600</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>D2</t>
         </is>
       </c>
     </row>
@@ -889,21 +889,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-2</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>8995</v>
+        <v>10598</v>
       </c>
       <c r="D13" t="n">
-        <v>23395</v>
+        <v>18004</v>
       </c>
       <c r="E13" t="n">
-        <v>14400</v>
+        <v>7406</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
@@ -913,21 +913,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-2</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>8995</v>
+        <v>18004</v>
       </c>
       <c r="D14" t="n">
-        <v>18595</v>
+        <v>24484</v>
       </c>
       <c r="E14" t="n">
-        <v>9600</v>
+        <v>6480</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>C3_1</t>
         </is>
       </c>
     </row>
@@ -937,21 +937,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10598</v>
+        <v>18004</v>
       </c>
       <c r="D15" t="n">
-        <v>18004</v>
+        <v>23188</v>
       </c>
       <c r="E15" t="n">
-        <v>7406</v>
+        <v>5184</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C3_1</t>
         </is>
       </c>
     </row>
@@ -961,21 +961,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>18004</v>
+        <v>24484</v>
       </c>
       <c r="D16" t="n">
-        <v>24484</v>
+        <v>36484</v>
       </c>
       <c r="E16" t="n">
-        <v>6480</v>
+        <v>12000</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>C4_1</t>
         </is>
       </c>
     </row>
@@ -985,21 +985,21 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>18004</v>
+        <v>24484</v>
       </c>
       <c r="D17" t="n">
-        <v>23188</v>
+        <v>38884</v>
       </c>
       <c r="E17" t="n">
-        <v>5184</v>
+        <v>14400</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>C4_1</t>
         </is>
       </c>
     </row>
@@ -1009,21 +1009,21 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-5</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23395</v>
+        <v>24909</v>
       </c>
       <c r="D18" t="n">
-        <v>28024</v>
+        <v>31081</v>
       </c>
       <c r="E18" t="n">
-        <v>4629</v>
+        <v>6172</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>E2</t>
         </is>
       </c>
     </row>
@@ -1033,21 +1033,21 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>24484</v>
+        <v>31596</v>
       </c>
       <c r="D19" t="n">
-        <v>36484</v>
+        <v>36225</v>
       </c>
       <c r="E19" t="n">
-        <v>12000</v>
+        <v>4629</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>D3</t>
         </is>
       </c>
     </row>
@@ -1057,21 +1057,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Precision Filling Machine1-3</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>24484</v>
+        <v>31630</v>
       </c>
       <c r="D20" t="n">
-        <v>38884</v>
+        <v>35333</v>
       </c>
       <c r="E20" t="n">
-        <v>14400</v>
+        <v>3703</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>B3</t>
         </is>
       </c>
     </row>
@@ -1081,21 +1081,21 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>24909</v>
+        <v>36744</v>
       </c>
       <c r="D21" t="n">
-        <v>31081</v>
+        <v>81744</v>
       </c>
       <c r="E21" t="n">
-        <v>6172</v>
+        <v>45000</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>D4</t>
         </is>
       </c>
     </row>
@@ -1105,21 +1105,21 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-3</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>31630</v>
+        <v>36744</v>
       </c>
       <c r="D22" t="n">
-        <v>35333</v>
+        <v>54744</v>
       </c>
       <c r="E22" t="n">
-        <v>3703</v>
+        <v>18000</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>D4</t>
         </is>
       </c>
     </row>
@@ -1129,21 +1129,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>36744</v>
+        <v>55259</v>
       </c>
       <c r="D23" t="n">
-        <v>81744</v>
+        <v>62459</v>
       </c>
       <c r="E23" t="n">
-        <v>45000</v>
+        <v>7200</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>E3</t>
         </is>
       </c>
     </row>
@@ -1153,21 +1153,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>36744</v>
+        <v>55259</v>
       </c>
       <c r="D24" t="n">
-        <v>54744</v>
+        <v>76859</v>
       </c>
       <c r="E24" t="n">
-        <v>18000</v>
+        <v>21600</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>E3</t>
         </is>
       </c>
     </row>
@@ -1181,17 +1181,17 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>55259</v>
+        <v>62884</v>
       </c>
       <c r="D25" t="n">
-        <v>62459</v>
+        <v>77284</v>
       </c>
       <c r="E25" t="n">
-        <v>7200</v>
+        <v>14400</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>C5_1</t>
         </is>
       </c>
     </row>
@@ -1201,21 +1201,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>55259</v>
+        <v>77284</v>
       </c>
       <c r="D26" t="n">
-        <v>76859</v>
+        <v>83764</v>
       </c>
       <c r="E26" t="n">
-        <v>21600</v>
+        <v>6480</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>C3_2</t>
         </is>
       </c>
     </row>
@@ -1225,21 +1225,21 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Automated Conveying Arm1-4</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>62884</v>
+        <v>77284</v>
       </c>
       <c r="D27" t="n">
-        <v>77284</v>
+        <v>82468</v>
       </c>
       <c r="E27" t="n">
-        <v>14400</v>
+        <v>5184</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C5_1</t>
+          <t>C3_2</t>
         </is>
       </c>
     </row>
@@ -1249,21 +1249,21 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>77284</v>
+        <v>81744</v>
       </c>
       <c r="D28" t="n">
-        <v>83764</v>
+        <v>99744</v>
       </c>
       <c r="E28" t="n">
-        <v>6480</v>
+        <v>18000</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>D5</t>
         </is>
       </c>
     </row>
@@ -1273,21 +1273,21 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>77284</v>
+        <v>83764</v>
       </c>
       <c r="D29" t="n">
-        <v>82468</v>
+        <v>95764</v>
       </c>
       <c r="E29" t="n">
-        <v>5184</v>
+        <v>12000</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>C4_2</t>
         </is>
       </c>
     </row>
@@ -1297,21 +1297,21 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>81744</v>
+        <v>83764</v>
       </c>
       <c r="D30" t="n">
-        <v>99744</v>
+        <v>98164</v>
       </c>
       <c r="E30" t="n">
-        <v>18000</v>
+        <v>14400</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>C4_2</t>
         </is>
       </c>
     </row>
@@ -1325,17 +1325,17 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>83764</v>
+        <v>96289</v>
       </c>
       <c r="D31" t="n">
-        <v>95764</v>
+        <v>114289</v>
       </c>
       <c r="E31" t="n">
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>A2</t>
         </is>
       </c>
     </row>
@@ -1345,21 +1345,21 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Industrial Cleaning Machine1-5</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>83764</v>
+        <v>96289</v>
       </c>
       <c r="D32" t="n">
-        <v>98164</v>
+        <v>103489</v>
       </c>
       <c r="E32" t="n">
-        <v>14400</v>
+        <v>7200</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>A2</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1660,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Precision Filling Machine1-2</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-3</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Industrial Cleaning Machine1-2</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-2</t>
+          <t>Automated Conveying Arm1-3</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1813,7 +1813,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-2</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1849,25 +1849,25 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Precision Filling Machine2-3</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10598</v>
+        <v>8995</v>
       </c>
       <c r="D9" t="n">
-        <v>18004</v>
+        <v>23395</v>
       </c>
       <c r="E9" t="n">
-        <v>7406</v>
+        <v>14400</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1876,17 +1876,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-2</t>
+          <t>Automated Conveying Arm1-2</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>10858</v>
+        <v>8995</v>
       </c>
       <c r="D10" t="n">
-        <v>25258</v>
+        <v>18595</v>
       </c>
       <c r="E10" t="n">
-        <v>14400</v>
+        <v>9600</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1903,21 +1903,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-2</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10858</v>
+        <v>10598</v>
       </c>
       <c r="D11" t="n">
-        <v>20458</v>
+        <v>18004</v>
       </c>
       <c r="E11" t="n">
-        <v>9600</v>
+        <v>7406</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -1930,21 +1930,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-2</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>13500</v>
+        <v>18004</v>
       </c>
       <c r="D12" t="n">
-        <v>27900</v>
+        <v>24484</v>
       </c>
       <c r="E12" t="n">
-        <v>14400</v>
+        <v>6480</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>C3_1</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -1957,17 +1957,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>18004</v>
       </c>
       <c r="D13" t="n">
-        <v>24484</v>
+        <v>23188</v>
       </c>
       <c r="E13" t="n">
-        <v>6480</v>
+        <v>5184</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1984,21 +1984,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>18004</v>
+        <v>24484</v>
       </c>
       <c r="D14" t="n">
-        <v>23188</v>
+        <v>36484</v>
       </c>
       <c r="E14" t="n">
-        <v>5184</v>
+        <v>12000</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>C4_1</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -2011,17 +2011,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>24484</v>
       </c>
       <c r="D15" t="n">
-        <v>36484</v>
+        <v>38884</v>
       </c>
       <c r="E15" t="n">
-        <v>12000</v>
+        <v>14400</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -2038,21 +2038,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>24484</v>
+        <v>24744</v>
       </c>
       <c r="D16" t="n">
-        <v>38884</v>
+        <v>29373</v>
       </c>
       <c r="E16" t="n">
-        <v>14400</v>
+        <v>4629</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -2065,25 +2065,25 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>25258</v>
+        <v>29373</v>
       </c>
       <c r="D17" t="n">
-        <v>29887</v>
+        <v>74373</v>
       </c>
       <c r="E17" t="n">
-        <v>4629</v>
+        <v>45000</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -2092,17 +2092,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>29887</v>
+        <v>29373</v>
       </c>
       <c r="D18" t="n">
-        <v>74887</v>
+        <v>47373</v>
       </c>
       <c r="E18" t="n">
-        <v>45000</v>
+        <v>18000</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -2110,7 +2110,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -2119,25 +2119,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>29887</v>
+        <v>38884</v>
       </c>
       <c r="D19" t="n">
-        <v>47887</v>
+        <v>53284</v>
       </c>
       <c r="E19" t="n">
-        <v>18000</v>
+        <v>14400</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>C5_1</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -2146,21 +2146,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>30402</v>
+        <v>39309</v>
       </c>
       <c r="D20" t="n">
-        <v>36574</v>
+        <v>53709</v>
       </c>
       <c r="E20" t="n">
-        <v>6172</v>
+        <v>14400</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -2173,25 +2173,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>38884</v>
+        <v>47823</v>
       </c>
       <c r="D21" t="n">
-        <v>53284</v>
+        <v>65823</v>
       </c>
       <c r="E21" t="n">
-        <v>14400</v>
+        <v>18000</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>C5_1</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2200,21 +2200,21 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>39434</v>
+        <v>53284</v>
       </c>
       <c r="D22" t="n">
-        <v>43754</v>
+        <v>59764</v>
       </c>
       <c r="E22" t="n">
-        <v>4320</v>
+        <v>6480</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>C3_2</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -2227,17 +2227,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>53284</v>
       </c>
       <c r="D23" t="n">
-        <v>59764</v>
+        <v>58468</v>
       </c>
       <c r="E23" t="n">
-        <v>6480</v>
+        <v>5184</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -2254,21 +2254,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-4</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>53284</v>
+        <v>54069</v>
       </c>
       <c r="D24" t="n">
-        <v>58468</v>
+        <v>58389</v>
       </c>
       <c r="E24" t="n">
-        <v>5184</v>
+        <v>4320</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -2281,25 +2281,25 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>Precision Filling Machine1-2</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>53709</v>
+        <v>59018</v>
       </c>
       <c r="D25" t="n">
-        <v>60909</v>
+        <v>86018</v>
       </c>
       <c r="E25" t="n">
-        <v>7200</v>
+        <v>27000</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -2308,21 +2308,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-4</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>53709</v>
+        <v>59018</v>
       </c>
       <c r="D26" t="n">
-        <v>75309</v>
+        <v>77018</v>
       </c>
       <c r="E26" t="n">
-        <v>21600</v>
+        <v>18000</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -2393,17 +2393,17 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>60314</v>
+        <v>60189</v>
       </c>
       <c r="D29" t="n">
-        <v>87314</v>
+        <v>66361</v>
       </c>
       <c r="E29" t="n">
-        <v>27000</v>
+        <v>6172</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -2416,25 +2416,25 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm2-4</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>60314</v>
+        <v>66523</v>
       </c>
       <c r="D30" t="n">
-        <v>78314</v>
+        <v>73723</v>
       </c>
       <c r="E30" t="n">
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -2443,21 +2443,21 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Industrial Cleaning Machine1-2</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>74164</v>
+        <v>66523</v>
       </c>
       <c r="D31" t="n">
-        <v>88564</v>
+        <v>88123</v>
       </c>
       <c r="E31" t="n">
-        <v>14400</v>
+        <v>21600</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C5_2</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -2474,17 +2474,17 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>74887</v>
+        <v>74164</v>
       </c>
       <c r="D32" t="n">
-        <v>92887</v>
+        <v>88564</v>
       </c>
       <c r="E32" t="n">
-        <v>18000</v>
+        <v>14400</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>C5_2</t>
         </is>
       </c>
       <c r="G32" t="n">
@@ -2497,21 +2497,21 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>88564</v>
+        <v>74373</v>
       </c>
       <c r="D33" t="n">
-        <v>95044</v>
+        <v>92373</v>
       </c>
       <c r="E33" t="n">
-        <v>6480</v>
+        <v>18000</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C3_3</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="G33" t="n">
@@ -2524,25 +2524,25 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Precision Filling Machine2-5</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>88564</v>
+        <v>86018</v>
       </c>
       <c r="D34" t="n">
-        <v>93748</v>
+        <v>89721</v>
       </c>
       <c r="E34" t="n">
-        <v>5184</v>
+        <v>3703</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C3_3</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
@@ -2551,21 +2551,21 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>89089</v>
+        <v>88564</v>
       </c>
       <c r="D35" t="n">
-        <v>107089</v>
+        <v>95044</v>
       </c>
       <c r="E35" t="n">
-        <v>18000</v>
+        <v>6480</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>C3_3</t>
         </is>
       </c>
       <c r="G35" t="n">
@@ -2578,25 +2578,25 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>92887</v>
+        <v>88564</v>
       </c>
       <c r="D36" t="n">
-        <v>118087</v>
+        <v>93748</v>
       </c>
       <c r="E36" t="n">
-        <v>25200</v>
+        <v>5184</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>C3_3</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -2609,17 +2609,17 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>95044</v>
+        <v>92373</v>
       </c>
       <c r="D37" t="n">
-        <v>107044</v>
+        <v>117573</v>
       </c>
       <c r="E37" t="n">
-        <v>12000</v>
+        <v>25200</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C4_3</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="G37" t="n">
@@ -2632,17 +2632,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>95044</v>
       </c>
       <c r="D38" t="n">
-        <v>109444</v>
+        <v>107044</v>
       </c>
       <c r="E38" t="n">
-        <v>14400</v>
+        <v>12000</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2650,7 +2650,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
@@ -2659,21 +2659,21 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>95594</v>
+        <v>95044</v>
       </c>
       <c r="D39" t="n">
-        <v>99297</v>
+        <v>109444</v>
       </c>
       <c r="E39" t="n">
-        <v>3703</v>
+        <v>14400</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>C4_3</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2704,7 +2704,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_8</t>
+          <t>Industrial Cleaning Machine1-2</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -2845,25 +2845,25 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-5</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>230</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>4550</v>
+        <v>5601</v>
       </c>
       <c r="E3" t="n">
-        <v>4320</v>
+        <v>5400</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -2872,21 +2872,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_5</t>
+          <t>Automated Conveying Arm1-3</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>230</v>
+        <v>201</v>
       </c>
       <c r="D4" t="n">
-        <v>10598</v>
+        <v>4521</v>
       </c>
       <c r="E4" t="n">
-        <v>10368</v>
+        <v>4320</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -2926,21 +2926,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="D6" t="n">
-        <v>5650</v>
+        <v>10598</v>
       </c>
       <c r="E6" t="n">
-        <v>5400</v>
+        <v>10368</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -2953,25 +2953,25 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm2-2</t>
+          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_1</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>250</v>
+        <v>310</v>
       </c>
       <c r="D7" t="n">
-        <v>4570</v>
+        <v>4630</v>
       </c>
       <c r="E7" t="n">
         <v>4320</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-1</t>
+          <t>Industrial Cleaning Machine2-4</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -3007,21 +3007,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-5</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4550</v>
+        <v>5650</v>
       </c>
       <c r="D9" t="n">
-        <v>31550</v>
+        <v>23650</v>
       </c>
       <c r="E9" t="n">
-        <v>27000</v>
+        <v>18000</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -3034,25 +3034,25 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm2-1</t>
+          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_6</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4550</v>
+        <v>5650</v>
       </c>
       <c r="D10" t="n">
-        <v>22550</v>
+        <v>12850</v>
       </c>
       <c r="E10" t="n">
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -3061,21 +3061,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5650</v>
+        <v>8995</v>
       </c>
       <c r="D11" t="n">
-        <v>23650</v>
+        <v>23395</v>
       </c>
       <c r="E11" t="n">
-        <v>18000</v>
+        <v>14400</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -3088,21 +3088,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-2</t>
+          <t>Automated Conveying Arm1-3</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5650</v>
+        <v>8995</v>
       </c>
       <c r="D12" t="n">
-        <v>12850</v>
+        <v>18595</v>
       </c>
       <c r="E12" t="n">
-        <v>7200</v>
+        <v>9600</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>New_PRECISION_FILLING_MACHINE_1_8</t>
+          <t>New_PRECISION_FILLING_MACHINE_2_13</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -3133,7 +3133,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -3142,25 +3142,25 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-4</t>
+          <t>Precision Filling Machine1-2</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10858</v>
+        <v>11148</v>
       </c>
       <c r="D14" t="n">
-        <v>25258</v>
+        <v>38148</v>
       </c>
       <c r="E14" t="n">
-        <v>14400</v>
+        <v>27000</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -3173,17 +3173,17 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10858</v>
+        <v>11148</v>
       </c>
       <c r="D15" t="n">
-        <v>20458</v>
+        <v>29148</v>
       </c>
       <c r="E15" t="n">
-        <v>9600</v>
+        <v>18000</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -3196,25 +3196,25 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>New_PRECISION_FILLING_MACHINE_1_0</t>
+          <t>New_PRECISION_FILLING_MACHINE_2_13</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14675</v>
+        <v>18004</v>
       </c>
       <c r="D16" t="n">
-        <v>20847</v>
+        <v>24484</v>
       </c>
       <c r="E16" t="n">
-        <v>6172</v>
+        <v>6480</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>C3_1</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -3223,17 +3223,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-3</t>
+          <t>Automated Conveying Arm2-4</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>18004</v>
       </c>
       <c r="D17" t="n">
-        <v>24484</v>
+        <v>23188</v>
       </c>
       <c r="E17" t="n">
-        <v>6480</v>
+        <v>5184</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -3250,25 +3250,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-2</t>
+          <t>Precision Filling Machine2-2</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>18004</v>
+        <v>23395</v>
       </c>
       <c r="D18" t="n">
-        <v>23188</v>
+        <v>28024</v>
       </c>
       <c r="E18" t="n">
-        <v>5184</v>
+        <v>4629</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -3277,21 +3277,21 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_2_4</t>
+          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_3</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20847</v>
+        <v>24484</v>
       </c>
       <c r="D19" t="n">
-        <v>28047</v>
+        <v>36484</v>
       </c>
       <c r="E19" t="n">
-        <v>7200</v>
+        <v>12000</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>C4_1</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -3304,21 +3304,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-4</t>
+          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_4</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>20847</v>
+        <v>24484</v>
       </c>
       <c r="D20" t="n">
-        <v>42447</v>
+        <v>38884</v>
       </c>
       <c r="E20" t="n">
-        <v>21600</v>
+        <v>14400</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>C4_1</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -3331,21 +3331,21 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_1_5</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>24484</v>
+        <v>28025</v>
       </c>
       <c r="D21" t="n">
-        <v>36484</v>
+        <v>73025</v>
       </c>
       <c r="E21" t="n">
-        <v>12000</v>
+        <v>45000</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -3358,25 +3358,25 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_3</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>24484</v>
+        <v>28025</v>
       </c>
       <c r="D22" t="n">
-        <v>38884</v>
+        <v>46025</v>
       </c>
       <c r="E22" t="n">
-        <v>14400</v>
+        <v>18000</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -3385,25 +3385,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Precision Filling Machine2-1</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>25258</v>
+        <v>38148</v>
       </c>
       <c r="D23" t="n">
-        <v>29887</v>
+        <v>41851</v>
       </c>
       <c r="E23" t="n">
-        <v>4629</v>
+        <v>3703</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -3412,21 +3412,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>29887</v>
+        <v>38884</v>
       </c>
       <c r="D24" t="n">
-        <v>74887</v>
+        <v>53284</v>
       </c>
       <c r="E24" t="n">
-        <v>45000</v>
+        <v>14400</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>C5_1</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -3439,21 +3439,21 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>29887</v>
+        <v>40352</v>
       </c>
       <c r="D25" t="n">
-        <v>47887</v>
+        <v>46524</v>
       </c>
       <c r="E25" t="n">
-        <v>18000</v>
+        <v>6172</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -3466,21 +3466,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-2</t>
+          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_2_5</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>31550</v>
+        <v>46539</v>
       </c>
       <c r="D26" t="n">
-        <v>35253</v>
+        <v>53739</v>
       </c>
       <c r="E26" t="n">
-        <v>3703</v>
+        <v>7200</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -3493,25 +3493,25 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_2_2</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>38884</v>
+        <v>46539</v>
       </c>
       <c r="D27" t="n">
-        <v>53284</v>
+        <v>68139</v>
       </c>
       <c r="E27" t="n">
-        <v>14400</v>
+        <v>21600</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C5_1</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -3520,21 +3520,21 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>44289</v>
+        <v>46840</v>
       </c>
       <c r="D28" t="n">
-        <v>62289</v>
+        <v>57640</v>
       </c>
       <c r="E28" t="n">
-        <v>18000</v>
+        <v>10800</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -3547,21 +3547,21 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-1</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>53284</v>
+        <v>46840</v>
       </c>
       <c r="D29" t="n">
-        <v>59764</v>
+        <v>59800</v>
       </c>
       <c r="E29" t="n">
-        <v>6480</v>
+        <v>12960</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -3574,17 +3574,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-4</t>
+          <t>New_PRECISION_FILLING_MACHINE_2_13</t>
         </is>
       </c>
       <c r="C30" t="n">
         <v>53284</v>
       </c>
       <c r="D30" t="n">
-        <v>58468</v>
+        <v>59764</v>
       </c>
       <c r="E30" t="n">
-        <v>5184</v>
+        <v>6480</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -3592,7 +3592,7 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -3601,21 +3601,21 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_2</t>
+          <t>New_AUTOMATED_CONVEYING_ARM_2_1</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>59764</v>
+        <v>53284</v>
       </c>
       <c r="D31" t="n">
-        <v>71764</v>
+        <v>58468</v>
       </c>
       <c r="E31" t="n">
-        <v>12000</v>
+        <v>5184</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>C3_2</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -3628,25 +3628,25 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_2_5</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>59764</v>
+        <v>54440</v>
       </c>
       <c r="D32" t="n">
-        <v>74164</v>
+        <v>72440</v>
       </c>
       <c r="E32" t="n">
-        <v>14400</v>
+        <v>18000</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -3655,21 +3655,21 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_2_4</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>74164</v>
+        <v>59764</v>
       </c>
       <c r="D33" t="n">
-        <v>88564</v>
+        <v>71764</v>
       </c>
       <c r="E33" t="n">
-        <v>14400</v>
+        <v>12000</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C5_2</t>
+          <t>C4_2</t>
         </is>
       </c>
       <c r="G33" t="n">
@@ -3682,21 +3682,21 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_7</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>74887</v>
+        <v>59764</v>
       </c>
       <c r="D34" t="n">
-        <v>92887</v>
+        <v>74164</v>
       </c>
       <c r="E34" t="n">
-        <v>18000</v>
+        <v>14400</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>C4_2</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -3709,25 +3709,25 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>New_PRECISION_FILLING_MACHINE_1_0</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>88564</v>
+        <v>73025</v>
       </c>
       <c r="D35" t="n">
-        <v>95044</v>
+        <v>91025</v>
       </c>
       <c r="E35" t="n">
-        <v>6480</v>
+        <v>18000</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C3_3</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -3736,25 +3736,25 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm2-4</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C36" t="n">
+        <v>74164</v>
+      </c>
+      <c r="D36" t="n">
         <v>88564</v>
       </c>
-      <c r="D36" t="n">
-        <v>93748</v>
-      </c>
       <c r="E36" t="n">
-        <v>5184</v>
+        <v>14400</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C3_3</t>
+          <t>C5_2</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -3763,25 +3763,25 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_1_5</t>
+          <t>New_PRECISION_FILLING_MACHINE_2_13</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>92887</v>
+        <v>88564</v>
       </c>
       <c r="D37" t="n">
-        <v>118087</v>
+        <v>95044</v>
       </c>
       <c r="E37" t="n">
-        <v>25200</v>
+        <v>6480</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>C3_3</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -3790,25 +3790,25 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_2</t>
+          <t>Automated Conveying Arm1-2</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>95044</v>
+        <v>88564</v>
       </c>
       <c r="D38" t="n">
-        <v>107044</v>
+        <v>93748</v>
       </c>
       <c r="E38" t="n">
-        <v>12000</v>
+        <v>5184</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C4_3</t>
+          <t>C3_3</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -3817,21 +3817,21 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-2</t>
+          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_3</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>95044</v>
+        <v>91025</v>
       </c>
       <c r="D39" t="n">
-        <v>109444</v>
+        <v>116225</v>
       </c>
       <c r="E39" t="n">
-        <v>14400</v>
+        <v>25200</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C4_3</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -3844,25 +3844,25 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_2</t>
+          <t>New_HIGH_SPEED_POLISHING_MACHINE_1_4</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>107674</v>
+        <v>95044</v>
       </c>
       <c r="D40" t="n">
-        <v>118474</v>
+        <v>107044</v>
       </c>
       <c r="E40" t="n">
-        <v>10800</v>
+        <v>12000</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>C4_3</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -3871,21 +3871,21 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_2_2</t>
+          <t>Industrial Cleaning Machine2-3</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>107674</v>
+        <v>95044</v>
       </c>
       <c r="D41" t="n">
-        <v>120634</v>
+        <v>109444</v>
       </c>
       <c r="E41" t="n">
-        <v>12960</v>
+        <v>14400</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>C4_3</t>
         </is>
       </c>
       <c r="G41" t="n">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -3916,7 +3916,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -3960,7 +3960,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -3970,7 +3970,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -3983,10 +3983,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -3999,7 +3999,7 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>采购费用500000/500000</t>
+          <t>采购费用475000/500000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final result tables and paper draft
</commit_message>
<xml_diff>
--- a/outputs/result_tables.xlsx
+++ b/outputs/result_tables.xlsx
@@ -841,21 +841,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-2</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8995</v>
+        <v>5600</v>
       </c>
       <c r="D11" t="n">
-        <v>23395</v>
+        <v>23600</v>
       </c>
       <c r="E11" t="n">
-        <v>14400</v>
+        <v>18000</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>A2</t>
         </is>
       </c>
     </row>
@@ -865,21 +865,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-2</t>
+          <t>Industrial Cleaning Machine1-5</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>8995</v>
+        <v>5600</v>
       </c>
       <c r="D12" t="n">
-        <v>18595</v>
+        <v>12800</v>
       </c>
       <c r="E12" t="n">
-        <v>9600</v>
+        <v>7200</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>A2</t>
         </is>
       </c>
     </row>
@@ -889,21 +889,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Precision Filling Machine1-2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10598</v>
+        <v>8995</v>
       </c>
       <c r="D13" t="n">
-        <v>18004</v>
+        <v>23395</v>
       </c>
       <c r="E13" t="n">
-        <v>7406</v>
+        <v>14400</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>D2</t>
         </is>
       </c>
     </row>
@@ -913,21 +913,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automated Conveying Arm1-2</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>18004</v>
+        <v>8995</v>
       </c>
       <c r="D14" t="n">
-        <v>24484</v>
+        <v>18595</v>
       </c>
       <c r="E14" t="n">
-        <v>6480</v>
+        <v>9600</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>D2</t>
         </is>
       </c>
     </row>
@@ -937,21 +937,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C15" t="n">
+        <v>10598</v>
+      </c>
+      <c r="D15" t="n">
         <v>18004</v>
       </c>
-      <c r="D15" t="n">
-        <v>23188</v>
-      </c>
       <c r="E15" t="n">
-        <v>5184</v>
+        <v>7406</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
@@ -961,21 +961,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C16" t="n">
+        <v>18004</v>
+      </c>
+      <c r="D16" t="n">
         <v>24484</v>
       </c>
-      <c r="D16" t="n">
-        <v>36484</v>
-      </c>
       <c r="E16" t="n">
-        <v>12000</v>
+        <v>6480</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>C3_1</t>
         </is>
       </c>
     </row>
@@ -985,21 +985,21 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>24484</v>
+        <v>18004</v>
       </c>
       <c r="D17" t="n">
-        <v>38884</v>
+        <v>23188</v>
       </c>
       <c r="E17" t="n">
-        <v>14400</v>
+        <v>5184</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>C3_1</t>
         </is>
       </c>
     </row>
@@ -1009,21 +1009,21 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Precision Filling Machine1-5</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>24909</v>
+        <v>23395</v>
       </c>
       <c r="D18" t="n">
-        <v>31081</v>
+        <v>28024</v>
       </c>
       <c r="E18" t="n">
-        <v>6172</v>
+        <v>4629</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>D3</t>
         </is>
       </c>
     </row>
@@ -1033,21 +1033,21 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>31596</v>
+        <v>24484</v>
       </c>
       <c r="D19" t="n">
-        <v>36225</v>
+        <v>36484</v>
       </c>
       <c r="E19" t="n">
-        <v>4629</v>
+        <v>12000</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>C4_1</t>
         </is>
       </c>
     </row>
@@ -1057,21 +1057,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-3</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>31630</v>
+        <v>24484</v>
       </c>
       <c r="D20" t="n">
-        <v>35333</v>
+        <v>38884</v>
       </c>
       <c r="E20" t="n">
-        <v>3703</v>
+        <v>14400</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>C4_1</t>
         </is>
       </c>
     </row>
@@ -1081,21 +1081,21 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>36744</v>
+        <v>24909</v>
       </c>
       <c r="D21" t="n">
-        <v>81744</v>
+        <v>31081</v>
       </c>
       <c r="E21" t="n">
-        <v>45000</v>
+        <v>6172</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>E2</t>
         </is>
       </c>
     </row>
@@ -1105,21 +1105,21 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Precision Filling Machine1-3</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>36744</v>
+        <v>31630</v>
       </c>
       <c r="D22" t="n">
-        <v>54744</v>
+        <v>35333</v>
       </c>
       <c r="E22" t="n">
-        <v>18000</v>
+        <v>3703</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>B3</t>
         </is>
       </c>
     </row>
@@ -1129,21 +1129,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>55259</v>
+        <v>36744</v>
       </c>
       <c r="D23" t="n">
-        <v>62459</v>
+        <v>81744</v>
       </c>
       <c r="E23" t="n">
-        <v>7200</v>
+        <v>45000</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>D4</t>
         </is>
       </c>
     </row>
@@ -1153,21 +1153,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>55259</v>
+        <v>36744</v>
       </c>
       <c r="D24" t="n">
-        <v>76859</v>
+        <v>54744</v>
       </c>
       <c r="E24" t="n">
-        <v>21600</v>
+        <v>18000</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>D4</t>
         </is>
       </c>
     </row>
@@ -1181,17 +1181,17 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>62884</v>
+        <v>55259</v>
       </c>
       <c r="D25" t="n">
-        <v>77284</v>
+        <v>62459</v>
       </c>
       <c r="E25" t="n">
-        <v>14400</v>
+        <v>7200</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>C5_1</t>
+          <t>E3</t>
         </is>
       </c>
     </row>
@@ -1201,21 +1201,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>77284</v>
+        <v>55259</v>
       </c>
       <c r="D26" t="n">
-        <v>83764</v>
+        <v>76859</v>
       </c>
       <c r="E26" t="n">
-        <v>6480</v>
+        <v>21600</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>E3</t>
         </is>
       </c>
     </row>
@@ -1225,21 +1225,21 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-4</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C27" t="n">
+        <v>62884</v>
+      </c>
+      <c r="D27" t="n">
         <v>77284</v>
       </c>
-      <c r="D27" t="n">
-        <v>82468</v>
-      </c>
       <c r="E27" t="n">
-        <v>5184</v>
+        <v>14400</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>C5_1</t>
         </is>
       </c>
     </row>
@@ -1249,21 +1249,21 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>81744</v>
+        <v>77284</v>
       </c>
       <c r="D28" t="n">
-        <v>99744</v>
+        <v>83764</v>
       </c>
       <c r="E28" t="n">
-        <v>18000</v>
+        <v>6480</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>C3_2</t>
         </is>
       </c>
     </row>
@@ -1273,21 +1273,21 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>83764</v>
+        <v>77284</v>
       </c>
       <c r="D29" t="n">
-        <v>95764</v>
+        <v>82468</v>
       </c>
       <c r="E29" t="n">
-        <v>12000</v>
+        <v>5184</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>C3_2</t>
         </is>
       </c>
     </row>
@@ -1297,21 +1297,21 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>83764</v>
+        <v>81744</v>
       </c>
       <c r="D30" t="n">
-        <v>98164</v>
+        <v>99744</v>
       </c>
       <c r="E30" t="n">
-        <v>14400</v>
+        <v>18000</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>D5</t>
         </is>
       </c>
     </row>
@@ -1325,17 +1325,17 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>96289</v>
+        <v>83764</v>
       </c>
       <c r="D31" t="n">
-        <v>114289</v>
+        <v>95764</v>
       </c>
       <c r="E31" t="n">
-        <v>18000</v>
+        <v>12000</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>C4_2</t>
         </is>
       </c>
     </row>
@@ -1345,21 +1345,21 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-5</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>96289</v>
+        <v>83764</v>
       </c>
       <c r="D32" t="n">
-        <v>103489</v>
+        <v>98164</v>
       </c>
       <c r="E32" t="n">
-        <v>7200</v>
+        <v>14400</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>C4_2</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Automated Conveying Arm1-3</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-2</t>
+          <t>Industrial Cleaning Machine1-3</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-3</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1768,25 +1768,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-3</t>
+          <t>Industrial Cleaning Machine2-5</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>355</v>
+        <v>275</v>
       </c>
       <c r="D6" t="n">
-        <v>8995</v>
+        <v>14675</v>
       </c>
       <c r="E6" t="n">
-        <v>8640</v>
+        <v>14400</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -1795,25 +1795,25 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>Industrial Cleaning Machine1-2</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5600</v>
+        <v>355</v>
       </c>
       <c r="D7" t="n">
-        <v>23600</v>
+        <v>8995</v>
       </c>
       <c r="E7" t="n">
-        <v>18000</v>
+        <v>8640</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1822,17 +1822,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>5600</v>
       </c>
       <c r="D8" t="n">
-        <v>12800</v>
+        <v>23600</v>
       </c>
       <c r="E8" t="n">
-        <v>7200</v>
+        <v>18000</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1849,25 +1849,25 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-3</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>8995</v>
+        <v>5600</v>
       </c>
       <c r="D9" t="n">
-        <v>23395</v>
+        <v>12800</v>
       </c>
       <c r="E9" t="n">
-        <v>14400</v>
+        <v>7200</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1876,17 +1876,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-2</t>
+          <t>Precision Filling Machine2-5</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>8995</v>
       </c>
       <c r="D10" t="n">
-        <v>18595</v>
+        <v>23395</v>
       </c>
       <c r="E10" t="n">
-        <v>9600</v>
+        <v>14400</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1894,7 +1894,7 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1903,25 +1903,25 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automated Conveying Arm2-4</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10598</v>
+        <v>8995</v>
       </c>
       <c r="D11" t="n">
-        <v>18004</v>
+        <v>18595</v>
       </c>
       <c r="E11" t="n">
-        <v>7406</v>
+        <v>9600</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -1930,25 +1930,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Precision Filling Machine2-4</t>
         </is>
       </c>
       <c r="C12" t="n">
+        <v>10598</v>
+      </c>
+      <c r="D12" t="n">
         <v>18004</v>
       </c>
-      <c r="D12" t="n">
-        <v>24484</v>
-      </c>
       <c r="E12" t="n">
-        <v>6480</v>
+        <v>7406</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1957,21 +1957,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Industrial Cleaning Machine1-3</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>18004</v>
+        <v>11148</v>
       </c>
       <c r="D13" t="n">
-        <v>23188</v>
+        <v>15468</v>
       </c>
       <c r="E13" t="n">
-        <v>5184</v>
+        <v>4320</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -1984,25 +1984,25 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine2-3</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>24484</v>
+        <v>14675</v>
       </c>
       <c r="D14" t="n">
-        <v>36484</v>
+        <v>20847</v>
       </c>
       <c r="E14" t="n">
-        <v>12000</v>
+        <v>6172</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -2011,21 +2011,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>24484</v>
+        <v>15468</v>
       </c>
       <c r="D15" t="n">
-        <v>38884</v>
+        <v>42468</v>
       </c>
       <c r="E15" t="n">
-        <v>14400</v>
+        <v>27000</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -2038,21 +2038,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automated Conveying Arm1-4</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>24744</v>
+        <v>15468</v>
       </c>
       <c r="D16" t="n">
-        <v>29373</v>
+        <v>33468</v>
       </c>
       <c r="E16" t="n">
-        <v>4629</v>
+        <v>18000</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -2065,21 +2065,21 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>Precision Filling Machine2-4</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>29373</v>
+        <v>18004</v>
       </c>
       <c r="D17" t="n">
-        <v>74373</v>
+        <v>24484</v>
       </c>
       <c r="E17" t="n">
-        <v>45000</v>
+        <v>6480</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>C3_1</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -2092,21 +2092,21 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>29373</v>
+        <v>18004</v>
       </c>
       <c r="D18" t="n">
-        <v>47373</v>
+        <v>23188</v>
       </c>
       <c r="E18" t="n">
-        <v>18000</v>
+        <v>5184</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>C3_1</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -2119,25 +2119,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>Precision Filling Machine1-5</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>38884</v>
+        <v>23395</v>
       </c>
       <c r="D19" t="n">
-        <v>53284</v>
+        <v>28024</v>
       </c>
       <c r="E19" t="n">
-        <v>14400</v>
+        <v>4629</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>C5_1</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2146,21 +2146,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>39309</v>
+        <v>24484</v>
       </c>
       <c r="D20" t="n">
-        <v>53709</v>
+        <v>36484</v>
       </c>
       <c r="E20" t="n">
-        <v>14400</v>
+        <v>12000</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>C4_1</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -2173,25 +2173,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Industrial Cleaning Machine2-4</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>47823</v>
+        <v>24484</v>
       </c>
       <c r="D21" t="n">
-        <v>65823</v>
+        <v>38884</v>
       </c>
       <c r="E21" t="n">
-        <v>18000</v>
+        <v>14400</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>C4_1</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -2200,25 +2200,25 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>53284</v>
+        <v>28024</v>
       </c>
       <c r="D22" t="n">
-        <v>59764</v>
+        <v>73024</v>
       </c>
       <c r="E22" t="n">
-        <v>6480</v>
+        <v>45000</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -2227,25 +2227,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>53284</v>
+        <v>28024</v>
       </c>
       <c r="D23" t="n">
-        <v>58468</v>
+        <v>46024</v>
       </c>
       <c r="E23" t="n">
-        <v>5184</v>
+        <v>18000</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -2254,21 +2254,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>54069</v>
+        <v>38884</v>
       </c>
       <c r="D24" t="n">
-        <v>58389</v>
+        <v>53284</v>
       </c>
       <c r="E24" t="n">
-        <v>4320</v>
+        <v>14400</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>C5_1</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -2281,21 +2281,21 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-2</t>
+          <t>Precision Filling Machine1-5</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>59018</v>
+        <v>42468</v>
       </c>
       <c r="D25" t="n">
-        <v>86018</v>
+        <v>46171</v>
       </c>
       <c r="E25" t="n">
-        <v>27000</v>
+        <v>3703</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -2308,21 +2308,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>59018</v>
+        <v>46839</v>
       </c>
       <c r="D26" t="n">
-        <v>77018</v>
+        <v>57639</v>
       </c>
       <c r="E26" t="n">
-        <v>18000</v>
+        <v>10800</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -2335,25 +2335,25 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>59764</v>
+        <v>46839</v>
       </c>
       <c r="D27" t="n">
-        <v>71764</v>
+        <v>59799</v>
       </c>
       <c r="E27" t="n">
-        <v>12000</v>
+        <v>12960</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -2362,21 +2362,21 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Precision Filling Machine1-5</t>
         </is>
       </c>
       <c r="C28" t="n">
+        <v>53284</v>
+      </c>
+      <c r="D28" t="n">
         <v>59764</v>
       </c>
-      <c r="D28" t="n">
-        <v>74164</v>
-      </c>
       <c r="E28" t="n">
-        <v>14400</v>
+        <v>6480</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>C3_2</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -2389,25 +2389,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automated Conveying Arm2-2</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>60189</v>
+        <v>53284</v>
       </c>
       <c r="D29" t="n">
-        <v>66361</v>
+        <v>58468</v>
       </c>
       <c r="E29" t="n">
-        <v>6172</v>
+        <v>5184</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>C3_2</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -2416,21 +2416,21 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>66523</v>
+        <v>59764</v>
       </c>
       <c r="D30" t="n">
-        <v>73723</v>
+        <v>71764</v>
       </c>
       <c r="E30" t="n">
-        <v>7200</v>
+        <v>12000</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>C4_2</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -2443,21 +2443,21 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-2</t>
+          <t>Industrial Cleaning Machine1-5</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>66523</v>
+        <v>59764</v>
       </c>
       <c r="D31" t="n">
-        <v>88123</v>
+        <v>74164</v>
       </c>
       <c r="E31" t="n">
-        <v>21600</v>
+        <v>14400</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>C4_2</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -2470,25 +2470,25 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>74164</v>
+        <v>73024</v>
       </c>
       <c r="D32" t="n">
-        <v>88564</v>
+        <v>91024</v>
       </c>
       <c r="E32" t="n">
-        <v>14400</v>
+        <v>18000</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C5_2</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -2497,25 +2497,25 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>74373</v>
+        <v>74164</v>
       </c>
       <c r="D33" t="n">
-        <v>92373</v>
+        <v>88564</v>
       </c>
       <c r="E33" t="n">
-        <v>18000</v>
+        <v>14400</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>C5_2</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -2524,21 +2524,21 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-5</t>
+          <t>Precision Filling Machine2-1</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>86018</v>
+        <v>88564</v>
       </c>
       <c r="D34" t="n">
-        <v>89721</v>
+        <v>95044</v>
       </c>
       <c r="E34" t="n">
-        <v>3703</v>
+        <v>6480</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>C3_3</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -2551,17 +2551,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automated Conveying Arm2-4</t>
         </is>
       </c>
       <c r="C35" t="n">
         <v>88564</v>
       </c>
       <c r="D35" t="n">
-        <v>95044</v>
+        <v>93748</v>
       </c>
       <c r="E35" t="n">
-        <v>6480</v>
+        <v>5184</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -2578,25 +2578,25 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>88564</v>
+        <v>89089</v>
       </c>
       <c r="D36" t="n">
-        <v>93748</v>
+        <v>107089</v>
       </c>
       <c r="E36" t="n">
-        <v>5184</v>
+        <v>18000</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C3_3</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -2605,14 +2605,14 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>92373</v>
+        <v>91024</v>
       </c>
       <c r="D37" t="n">
-        <v>117573</v>
+        <v>116224</v>
       </c>
       <c r="E37" t="n">
         <v>25200</v>
@@ -2623,7 +2623,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -2632,25 +2632,25 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>95044</v>
+        <v>91539</v>
       </c>
       <c r="D38" t="n">
-        <v>107044</v>
+        <v>98739</v>
       </c>
       <c r="E38" t="n">
-        <v>12000</v>
+        <v>7200</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C4_3</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -2659,21 +2659,21 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Industrial Cleaning Machine1-5</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>95044</v>
+        <v>91539</v>
       </c>
       <c r="D39" t="n">
-        <v>109444</v>
+        <v>113139</v>
       </c>
       <c r="E39" t="n">
-        <v>14400</v>
+        <v>21600</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C4_3</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -2686,25 +2686,25 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>107594</v>
+        <v>95044</v>
       </c>
       <c r="D40" t="n">
-        <v>118394</v>
+        <v>107044</v>
       </c>
       <c r="E40" t="n">
-        <v>10800</v>
+        <v>12000</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>C4_3</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -2713,25 +2713,25 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>107594</v>
+        <v>95044</v>
       </c>
       <c r="D41" t="n">
-        <v>120554</v>
+        <v>109444</v>
       </c>
       <c r="E41" t="n">
-        <v>12960</v>
+        <v>14400</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>C4_3</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -2758,7 +2758,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2818,25 +2818,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-2</t>
+          <t>Industrial Cleaning Machine2-1</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="D2" t="n">
-        <v>14600</v>
+        <v>4550</v>
       </c>
       <c r="E2" t="n">
-        <v>14400</v>
+        <v>4320</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -2845,21 +2845,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Industrial Cleaning Machine1-2</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>201</v>
+        <v>230</v>
       </c>
       <c r="D3" t="n">
-        <v>5601</v>
+        <v>10598</v>
       </c>
       <c r="E3" t="n">
-        <v>5400</v>
+        <v>10368</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -2872,21 +2872,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-3</t>
+          <t>New_AUTOMATED_CONVEYING_ARM_1_9</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>201</v>
+        <v>230</v>
       </c>
       <c r="D4" t="n">
-        <v>4521</v>
+        <v>10598</v>
       </c>
       <c r="E4" t="n">
-        <v>4320</v>
+        <v>10368</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -2899,25 +2899,25 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>New_PRECISION_FILLING_MACHINE_2_0</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="D5" t="n">
-        <v>10598</v>
+        <v>5650</v>
       </c>
       <c r="E5" t="n">
-        <v>10368</v>
+        <v>5400</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -2926,25 +2926,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Automated Conveying Arm2-1</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="D6" t="n">
-        <v>10598</v>
+        <v>4570</v>
       </c>
       <c r="E6" t="n">
-        <v>10368</v>
+        <v>4320</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -2953,25 +2953,25 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_1</t>
+          <t>Industrial Cleaning Machine2-4</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>310</v>
+        <v>340</v>
       </c>
       <c r="D7" t="n">
-        <v>4630</v>
+        <v>8980</v>
       </c>
       <c r="E7" t="n">
-        <v>4320</v>
+        <v>8640</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -2980,21 +2980,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-4</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>340</v>
+        <v>5650</v>
       </c>
       <c r="D8" t="n">
-        <v>8980</v>
+        <v>23650</v>
       </c>
       <c r="E8" t="n">
-        <v>8640</v>
+        <v>18000</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -3007,17 +3007,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>Industrial Cleaning Machine2-3</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>5650</v>
       </c>
       <c r="D9" t="n">
-        <v>23650</v>
+        <v>12850</v>
       </c>
       <c r="E9" t="n">
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -3034,25 +3034,25 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_6</t>
+          <t>Precision Filling Machine2-1</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5650</v>
+        <v>8980</v>
       </c>
       <c r="D10" t="n">
-        <v>12850</v>
+        <v>23380</v>
       </c>
       <c r="E10" t="n">
-        <v>7200</v>
+        <v>14400</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -3061,17 +3061,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automated Conveying Arm1-3</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8995</v>
+        <v>8980</v>
       </c>
       <c r="D11" t="n">
-        <v>23395</v>
+        <v>18580</v>
       </c>
       <c r="E11" t="n">
-        <v>14400</v>
+        <v>9600</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -3088,25 +3088,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-3</t>
+          <t>Industrial Cleaning Machine2-4</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>8995</v>
+        <v>9495</v>
       </c>
       <c r="D12" t="n">
-        <v>18595</v>
+        <v>23895</v>
       </c>
       <c r="E12" t="n">
-        <v>9600</v>
+        <v>14400</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>New_PRECISION_FILLING_MACHINE_2_13</t>
+          <t>Precision Filling Machine2-4</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-2</t>
+          <t>Precision Filling Machine2-3</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -3160,7 +3160,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -3169,7 +3169,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>New_AUTOMATED_CONVEYING_ARM_1_9</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>New_PRECISION_FILLING_MACHINE_2_13</t>
+          <t>Precision Filling Machine1-5</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -3214,7 +3214,7 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm2-4</t>
+          <t>Automated Conveying Arm2-2</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -3250,14 +3250,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-2</t>
+          <t>Precision Filling Machine2-5</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23395</v>
+        <v>23380</v>
       </c>
       <c r="D18" t="n">
-        <v>28024</v>
+        <v>28009</v>
       </c>
       <c r="E18" t="n">
         <v>4629</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_3</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_4</t>
+          <t>Industrial Cleaning Machine2-3</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -3322,7 +3322,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -3331,21 +3331,21 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine1-5</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>28025</v>
+        <v>24909</v>
       </c>
       <c r="D21" t="n">
-        <v>73025</v>
+        <v>31081</v>
       </c>
       <c r="E21" t="n">
-        <v>45000</v>
+        <v>6172</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -3358,17 +3358,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_4</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>28025</v>
+        <v>28009</v>
       </c>
       <c r="D22" t="n">
-        <v>46025</v>
+        <v>73009</v>
       </c>
       <c r="E22" t="n">
-        <v>18000</v>
+        <v>45000</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -3385,21 +3385,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-1</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>38148</v>
+        <v>28009</v>
       </c>
       <c r="D23" t="n">
-        <v>41851</v>
+        <v>46009</v>
       </c>
       <c r="E23" t="n">
-        <v>3703</v>
+        <v>18000</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -3412,21 +3412,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Precision Filling Machine1-5</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>38884</v>
+        <v>38148</v>
       </c>
       <c r="D24" t="n">
-        <v>53284</v>
+        <v>41851</v>
       </c>
       <c r="E24" t="n">
-        <v>14400</v>
+        <v>3703</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>C5_1</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -3439,21 +3439,21 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_4</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>40352</v>
+        <v>38884</v>
       </c>
       <c r="D25" t="n">
-        <v>46524</v>
+        <v>53284</v>
       </c>
       <c r="E25" t="n">
-        <v>6172</v>
+        <v>14400</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>C5_1</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -3466,21 +3466,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_2_5</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>46539</v>
+        <v>46459</v>
       </c>
       <c r="D26" t="n">
-        <v>53739</v>
+        <v>64459</v>
       </c>
       <c r="E26" t="n">
-        <v>7200</v>
+        <v>18000</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -3493,25 +3493,25 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Precision Filling Machine2-5</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>46539</v>
+        <v>53284</v>
       </c>
       <c r="D27" t="n">
-        <v>68139</v>
+        <v>59764</v>
       </c>
       <c r="E27" t="n">
-        <v>21600</v>
+        <v>6480</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>C3_2</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -3520,25 +3520,25 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>New_AUTOMATED_CONVEYING_ARM_1_9</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>46840</v>
+        <v>53284</v>
       </c>
       <c r="D28" t="n">
-        <v>57640</v>
+        <v>58468</v>
       </c>
       <c r="E28" t="n">
-        <v>10800</v>
+        <v>5184</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>C3_2</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -3547,21 +3547,21 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_2</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>46840</v>
+        <v>59764</v>
       </c>
       <c r="D29" t="n">
-        <v>59800</v>
+        <v>71764</v>
       </c>
       <c r="E29" t="n">
-        <v>12960</v>
+        <v>12000</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>C4_2</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -3574,21 +3574,21 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>New_PRECISION_FILLING_MACHINE_2_13</t>
+          <t>Industrial Cleaning Machine2-4</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>53284</v>
+        <v>59764</v>
       </c>
       <c r="D30" t="n">
-        <v>59764</v>
+        <v>74164</v>
       </c>
       <c r="E30" t="n">
-        <v>6480</v>
+        <v>14400</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>C4_2</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -3601,21 +3601,21 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>New_AUTOMATED_CONVEYING_ARM_2_1</t>
+          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_2</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>53284</v>
+        <v>72314</v>
       </c>
       <c r="D31" t="n">
-        <v>58468</v>
+        <v>83114</v>
       </c>
       <c r="E31" t="n">
-        <v>5184</v>
+        <v>10800</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -3628,25 +3628,25 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_2_5</t>
+          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_1</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>54440</v>
+        <v>72314</v>
       </c>
       <c r="D32" t="n">
-        <v>72440</v>
+        <v>85274</v>
       </c>
       <c r="E32" t="n">
-        <v>18000</v>
+        <v>12960</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -3655,25 +3655,25 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_5</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>59764</v>
+        <v>73009</v>
       </c>
       <c r="D33" t="n">
-        <v>71764</v>
+        <v>91009</v>
       </c>
       <c r="E33" t="n">
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -3682,21 +3682,21 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_7</t>
+          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_4</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>59764</v>
+        <v>74164</v>
       </c>
       <c r="D34" t="n">
-        <v>74164</v>
+        <v>88564</v>
       </c>
       <c r="E34" t="n">
         <v>14400</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>C5_2</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -3709,21 +3709,21 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>New_PRECISION_FILLING_MACHINE_2_0</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>73025</v>
+        <v>88564</v>
       </c>
       <c r="D35" t="n">
-        <v>91025</v>
+        <v>95044</v>
       </c>
       <c r="E35" t="n">
-        <v>18000</v>
+        <v>6480</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>C3_3</t>
         </is>
       </c>
       <c r="G35" t="n">
@@ -3736,25 +3736,25 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Automated Conveying Arm2-4</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>74164</v>
+        <v>88564</v>
       </c>
       <c r="D36" t="n">
-        <v>88564</v>
+        <v>93748</v>
       </c>
       <c r="E36" t="n">
-        <v>14400</v>
+        <v>5184</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C5_2</t>
+          <t>C3_3</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -3763,25 +3763,25 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>New_PRECISION_FILLING_MACHINE_2_13</t>
+          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_4</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>88564</v>
+        <v>88989</v>
       </c>
       <c r="D37" t="n">
-        <v>95044</v>
+        <v>96189</v>
       </c>
       <c r="E37" t="n">
-        <v>6480</v>
+        <v>7200</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C3_3</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -3790,21 +3790,21 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-2</t>
+          <t>Industrial Cleaning Machine1-5</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>88564</v>
+        <v>88989</v>
       </c>
       <c r="D38" t="n">
-        <v>93748</v>
+        <v>110589</v>
       </c>
       <c r="E38" t="n">
-        <v>5184</v>
+        <v>21600</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C3_3</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="G38" t="n">
@@ -3817,14 +3817,14 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_3</t>
+          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_2</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>91025</v>
+        <v>91009</v>
       </c>
       <c r="D39" t="n">
-        <v>116225</v>
+        <v>116209</v>
       </c>
       <c r="E39" t="n">
         <v>25200</v>
@@ -3844,7 +3844,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_1_4</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_5</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -3916,7 +3916,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3957,10 +3957,10 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
         <v>0</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -3970,7 +3970,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -3996,10 +3996,10 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="n">
         <v>0</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -4009,10 +4009,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Generate final paper draft and result tables
</commit_message>
<xml_diff>
--- a/outputs/result_tables.xlsx
+++ b/outputs/result_tables.xlsx
@@ -841,21 +841,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine1-2</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5600</v>
+        <v>8995</v>
       </c>
       <c r="D11" t="n">
-        <v>23600</v>
+        <v>23395</v>
       </c>
       <c r="E11" t="n">
-        <v>18000</v>
+        <v>14400</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>D2</t>
         </is>
       </c>
     </row>
@@ -865,21 +865,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-5</t>
+          <t>Automated Conveying Arm1-2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5600</v>
+        <v>8995</v>
       </c>
       <c r="D12" t="n">
-        <v>12800</v>
+        <v>18595</v>
       </c>
       <c r="E12" t="n">
-        <v>7200</v>
+        <v>9600</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>D2</t>
         </is>
       </c>
     </row>
@@ -889,21 +889,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-2</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>8995</v>
+        <v>10598</v>
       </c>
       <c r="D13" t="n">
-        <v>23395</v>
+        <v>18004</v>
       </c>
       <c r="E13" t="n">
-        <v>14400</v>
+        <v>7406</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
@@ -913,21 +913,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-2</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>8995</v>
+        <v>18004</v>
       </c>
       <c r="D14" t="n">
-        <v>18595</v>
+        <v>24484</v>
       </c>
       <c r="E14" t="n">
-        <v>9600</v>
+        <v>6480</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>C3_1</t>
         </is>
       </c>
     </row>
@@ -937,21 +937,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10598</v>
+        <v>18004</v>
       </c>
       <c r="D15" t="n">
-        <v>18004</v>
+        <v>23188</v>
       </c>
       <c r="E15" t="n">
-        <v>7406</v>
+        <v>5184</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C3_1</t>
         </is>
       </c>
     </row>
@@ -961,21 +961,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>18004</v>
+        <v>24484</v>
       </c>
       <c r="D16" t="n">
-        <v>24484</v>
+        <v>36484</v>
       </c>
       <c r="E16" t="n">
-        <v>6480</v>
+        <v>12000</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>C4_1</t>
         </is>
       </c>
     </row>
@@ -985,21 +985,21 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>18004</v>
+        <v>24484</v>
       </c>
       <c r="D17" t="n">
-        <v>23188</v>
+        <v>38884</v>
       </c>
       <c r="E17" t="n">
-        <v>5184</v>
+        <v>14400</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>C4_1</t>
         </is>
       </c>
     </row>
@@ -1009,21 +1009,21 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-5</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23395</v>
+        <v>24909</v>
       </c>
       <c r="D18" t="n">
-        <v>28024</v>
+        <v>31081</v>
       </c>
       <c r="E18" t="n">
-        <v>4629</v>
+        <v>6172</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>E2</t>
         </is>
       </c>
     </row>
@@ -1033,21 +1033,21 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>24484</v>
+        <v>31596</v>
       </c>
       <c r="D19" t="n">
-        <v>36484</v>
+        <v>36225</v>
       </c>
       <c r="E19" t="n">
-        <v>12000</v>
+        <v>4629</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>D3</t>
         </is>
       </c>
     </row>
@@ -1057,21 +1057,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Precision Filling Machine1-3</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>24484</v>
+        <v>31630</v>
       </c>
       <c r="D20" t="n">
-        <v>38884</v>
+        <v>35333</v>
       </c>
       <c r="E20" t="n">
-        <v>14400</v>
+        <v>3703</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>B3</t>
         </is>
       </c>
     </row>
@@ -1081,21 +1081,21 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>24909</v>
+        <v>36744</v>
       </c>
       <c r="D21" t="n">
-        <v>31081</v>
+        <v>81744</v>
       </c>
       <c r="E21" t="n">
-        <v>6172</v>
+        <v>45000</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>D4</t>
         </is>
       </c>
     </row>
@@ -1105,21 +1105,21 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-3</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>31630</v>
+        <v>36744</v>
       </c>
       <c r="D22" t="n">
-        <v>35333</v>
+        <v>54744</v>
       </c>
       <c r="E22" t="n">
-        <v>3703</v>
+        <v>18000</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>D4</t>
         </is>
       </c>
     </row>
@@ -1129,21 +1129,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>36744</v>
+        <v>55259</v>
       </c>
       <c r="D23" t="n">
-        <v>81744</v>
+        <v>62459</v>
       </c>
       <c r="E23" t="n">
-        <v>45000</v>
+        <v>7200</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>E3</t>
         </is>
       </c>
     </row>
@@ -1153,21 +1153,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>36744</v>
+        <v>55259</v>
       </c>
       <c r="D24" t="n">
-        <v>54744</v>
+        <v>76859</v>
       </c>
       <c r="E24" t="n">
-        <v>18000</v>
+        <v>21600</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>E3</t>
         </is>
       </c>
     </row>
@@ -1181,17 +1181,17 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>55259</v>
+        <v>62884</v>
       </c>
       <c r="D25" t="n">
-        <v>62459</v>
+        <v>77284</v>
       </c>
       <c r="E25" t="n">
-        <v>7200</v>
+        <v>14400</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>C5_1</t>
         </is>
       </c>
     </row>
@@ -1201,21 +1201,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>55259</v>
+        <v>77284</v>
       </c>
       <c r="D26" t="n">
-        <v>76859</v>
+        <v>83764</v>
       </c>
       <c r="E26" t="n">
-        <v>21600</v>
+        <v>6480</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>C3_2</t>
         </is>
       </c>
     </row>
@@ -1225,21 +1225,21 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Automated Conveying Arm1-4</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>62884</v>
+        <v>77284</v>
       </c>
       <c r="D27" t="n">
-        <v>77284</v>
+        <v>82468</v>
       </c>
       <c r="E27" t="n">
-        <v>14400</v>
+        <v>5184</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C5_1</t>
+          <t>C3_2</t>
         </is>
       </c>
     </row>
@@ -1249,21 +1249,21 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>77284</v>
+        <v>81744</v>
       </c>
       <c r="D28" t="n">
-        <v>83764</v>
+        <v>99744</v>
       </c>
       <c r="E28" t="n">
-        <v>6480</v>
+        <v>18000</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>D5</t>
         </is>
       </c>
     </row>
@@ -1273,21 +1273,21 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>77284</v>
+        <v>83764</v>
       </c>
       <c r="D29" t="n">
-        <v>82468</v>
+        <v>95764</v>
       </c>
       <c r="E29" t="n">
-        <v>5184</v>
+        <v>12000</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>C4_2</t>
         </is>
       </c>
     </row>
@@ -1297,21 +1297,21 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>81744</v>
+        <v>83764</v>
       </c>
       <c r="D30" t="n">
-        <v>99744</v>
+        <v>98164</v>
       </c>
       <c r="E30" t="n">
-        <v>18000</v>
+        <v>14400</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>C4_2</t>
         </is>
       </c>
     </row>
@@ -1325,17 +1325,17 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>83764</v>
+        <v>96289</v>
       </c>
       <c r="D31" t="n">
-        <v>95764</v>
+        <v>114289</v>
       </c>
       <c r="E31" t="n">
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>A2</t>
         </is>
       </c>
     </row>
@@ -1345,21 +1345,21 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Industrial Cleaning Machine1-5</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>83764</v>
+        <v>96289</v>
       </c>
       <c r="D32" t="n">
-        <v>98164</v>
+        <v>103489</v>
       </c>
       <c r="E32" t="n">
-        <v>14400</v>
+        <v>7200</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>A2</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1660,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-2</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-3</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-3</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Automated Conveying Arm1-2</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1768,25 +1768,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-5</t>
+          <t>Industrial Cleaning Machine1-2</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>275</v>
+        <v>355</v>
       </c>
       <c r="D6" t="n">
-        <v>14675</v>
+        <v>8995</v>
       </c>
       <c r="E6" t="n">
-        <v>14400</v>
+        <v>8640</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1795,21 +1795,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-2</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>355</v>
+        <v>10598</v>
       </c>
       <c r="D7" t="n">
-        <v>8995</v>
+        <v>18004</v>
       </c>
       <c r="E7" t="n">
-        <v>8640</v>
+        <v>7406</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -1822,21 +1822,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine1-2</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5600</v>
+        <v>10858</v>
       </c>
       <c r="D8" t="n">
-        <v>23600</v>
+        <v>25258</v>
       </c>
       <c r="E8" t="n">
-        <v>18000</v>
+        <v>14400</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -1849,21 +1849,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>Automated Conveying Arm1-2</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5600</v>
+        <v>10858</v>
       </c>
       <c r="D9" t="n">
-        <v>12800</v>
+        <v>20458</v>
       </c>
       <c r="E9" t="n">
-        <v>7200</v>
+        <v>9600</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -1876,21 +1876,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-5</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>8995</v>
+        <v>11123</v>
       </c>
       <c r="D10" t="n">
-        <v>23395</v>
+        <v>29123</v>
       </c>
       <c r="E10" t="n">
-        <v>14400</v>
+        <v>18000</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -1903,25 +1903,25 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm2-4</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8995</v>
+        <v>11123</v>
       </c>
       <c r="D11" t="n">
-        <v>18595</v>
+        <v>18323</v>
       </c>
       <c r="E11" t="n">
-        <v>9600</v>
+        <v>7200</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1930,25 +1930,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-4</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10598</v>
+        <v>18004</v>
       </c>
       <c r="D12" t="n">
-        <v>18004</v>
+        <v>24484</v>
       </c>
       <c r="E12" t="n">
-        <v>7406</v>
+        <v>6480</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C3_1</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1957,21 +1957,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-3</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>11148</v>
+        <v>18004</v>
       </c>
       <c r="D13" t="n">
-        <v>15468</v>
+        <v>23188</v>
       </c>
       <c r="E13" t="n">
-        <v>4320</v>
+        <v>5184</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>C3_1</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -1984,25 +1984,25 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-3</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>14675</v>
+        <v>24484</v>
       </c>
       <c r="D14" t="n">
-        <v>20847</v>
+        <v>36484</v>
       </c>
       <c r="E14" t="n">
-        <v>6172</v>
+        <v>12000</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>C4_1</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2011,21 +2011,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>15468</v>
+        <v>24484</v>
       </c>
       <c r="D15" t="n">
-        <v>42468</v>
+        <v>38884</v>
       </c>
       <c r="E15" t="n">
-        <v>27000</v>
+        <v>14400</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>C4_1</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -2038,21 +2038,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-4</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15468</v>
+        <v>25258</v>
       </c>
       <c r="D16" t="n">
-        <v>33468</v>
+        <v>29887</v>
       </c>
       <c r="E16" t="n">
-        <v>18000</v>
+        <v>4629</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -2065,21 +2065,21 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-4</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>18004</v>
+        <v>29887</v>
       </c>
       <c r="D17" t="n">
-        <v>24484</v>
+        <v>74887</v>
       </c>
       <c r="E17" t="n">
-        <v>6480</v>
+        <v>45000</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -2092,21 +2092,21 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>18004</v>
+        <v>29887</v>
       </c>
       <c r="D18" t="n">
-        <v>23188</v>
+        <v>47887</v>
       </c>
       <c r="E18" t="n">
-        <v>5184</v>
+        <v>18000</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -2119,25 +2119,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-5</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>23395</v>
+        <v>38884</v>
       </c>
       <c r="D19" t="n">
-        <v>28024</v>
+        <v>53284</v>
       </c>
       <c r="E19" t="n">
-        <v>4629</v>
+        <v>14400</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>C5_1</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -2146,21 +2146,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>24484</v>
+        <v>39309</v>
       </c>
       <c r="D20" t="n">
-        <v>36484</v>
+        <v>53709</v>
       </c>
       <c r="E20" t="n">
-        <v>12000</v>
+        <v>14400</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -2173,25 +2173,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-4</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>24484</v>
+        <v>53284</v>
       </c>
       <c r="D21" t="n">
-        <v>38884</v>
+        <v>59764</v>
       </c>
       <c r="E21" t="n">
-        <v>14400</v>
+        <v>6480</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>C3_2</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2200,25 +2200,25 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>28024</v>
+        <v>53284</v>
       </c>
       <c r="D22" t="n">
-        <v>73024</v>
+        <v>58468</v>
       </c>
       <c r="E22" t="n">
-        <v>45000</v>
+        <v>5184</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>C3_2</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -2231,17 +2231,17 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>28024</v>
+        <v>53809</v>
       </c>
       <c r="D23" t="n">
-        <v>46024</v>
+        <v>71809</v>
       </c>
       <c r="E23" t="n">
         <v>18000</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -2254,21 +2254,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>38884</v>
+        <v>59764</v>
       </c>
       <c r="D24" t="n">
-        <v>53284</v>
+        <v>71764</v>
       </c>
       <c r="E24" t="n">
-        <v>14400</v>
+        <v>12000</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>C5_1</t>
+          <t>C4_2</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -2281,21 +2281,21 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-5</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>42468</v>
+        <v>59764</v>
       </c>
       <c r="D25" t="n">
-        <v>46171</v>
+        <v>74164</v>
       </c>
       <c r="E25" t="n">
-        <v>3703</v>
+        <v>14400</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>C4_2</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -2308,21 +2308,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>46839</v>
+        <v>60189</v>
       </c>
       <c r="D26" t="n">
-        <v>57639</v>
+        <v>66361</v>
       </c>
       <c r="E26" t="n">
-        <v>10800</v>
+        <v>6172</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -2335,25 +2335,25 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>46839</v>
+        <v>74164</v>
       </c>
       <c r="D27" t="n">
-        <v>59799</v>
+        <v>88564</v>
       </c>
       <c r="E27" t="n">
-        <v>12960</v>
+        <v>14400</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>C5_2</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -2362,21 +2362,21 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-5</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>53284</v>
+        <v>74714</v>
       </c>
       <c r="D28" t="n">
-        <v>59764</v>
+        <v>79034</v>
       </c>
       <c r="E28" t="n">
-        <v>6480</v>
+        <v>4320</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -2389,21 +2389,21 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm2-2</t>
+          <t>Automatic Sensing Multi-Function Machine2-1</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>53284</v>
+        <v>74887</v>
       </c>
       <c r="D29" t="n">
-        <v>58468</v>
+        <v>92887</v>
       </c>
       <c r="E29" t="n">
-        <v>5184</v>
+        <v>18000</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -2416,21 +2416,21 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Precision Filling Machine1-2</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>59764</v>
+        <v>79034</v>
       </c>
       <c r="D30" t="n">
-        <v>71764</v>
+        <v>106034</v>
       </c>
       <c r="E30" t="n">
-        <v>12000</v>
+        <v>27000</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -2443,21 +2443,21 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-5</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>59764</v>
+        <v>79034</v>
       </c>
       <c r="D31" t="n">
-        <v>74164</v>
+        <v>97034</v>
       </c>
       <c r="E31" t="n">
-        <v>14400</v>
+        <v>18000</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -2470,25 +2470,25 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Precision Filling Machine2-2</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>73024</v>
+        <v>88564</v>
       </c>
       <c r="D32" t="n">
-        <v>91024</v>
+        <v>95044</v>
       </c>
       <c r="E32" t="n">
-        <v>18000</v>
+        <v>6480</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>C3_3</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -2497,25 +2497,25 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>Automated Conveying Arm1-3</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>74164</v>
+        <v>88564</v>
       </c>
       <c r="D33" t="n">
-        <v>88564</v>
+        <v>93748</v>
       </c>
       <c r="E33" t="n">
-        <v>14400</v>
+        <v>5184</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C5_2</t>
+          <t>C3_3</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -2524,25 +2524,25 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>88564</v>
+        <v>88989</v>
       </c>
       <c r="D34" t="n">
-        <v>95044</v>
+        <v>96189</v>
       </c>
       <c r="E34" t="n">
-        <v>6480</v>
+        <v>7200</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C3_3</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -2551,25 +2551,25 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm2-4</t>
+          <t>Industrial Cleaning Machine1-2</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>88564</v>
+        <v>88989</v>
       </c>
       <c r="D35" t="n">
-        <v>93748</v>
+        <v>110589</v>
       </c>
       <c r="E35" t="n">
-        <v>5184</v>
+        <v>21600</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C3_3</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -2578,21 +2578,21 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>89089</v>
+        <v>92887</v>
       </c>
       <c r="D36" t="n">
-        <v>107089</v>
+        <v>118087</v>
       </c>
       <c r="E36" t="n">
-        <v>18000</v>
+        <v>25200</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="G36" t="n">
@@ -2605,25 +2605,25 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>91024</v>
+        <v>95044</v>
       </c>
       <c r="D37" t="n">
-        <v>116224</v>
+        <v>107044</v>
       </c>
       <c r="E37" t="n">
-        <v>25200</v>
+        <v>12000</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>C4_3</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -2632,21 +2632,21 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine1-1</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>91539</v>
+        <v>95044</v>
       </c>
       <c r="D38" t="n">
-        <v>98739</v>
+        <v>109444</v>
       </c>
       <c r="E38" t="n">
-        <v>7200</v>
+        <v>14400</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>C4_3</t>
         </is>
       </c>
       <c r="G38" t="n">
@@ -2659,21 +2659,21 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-5</t>
+          <t>Precision Filling Machine1-1</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>91539</v>
+        <v>106034</v>
       </c>
       <c r="D39" t="n">
-        <v>113139</v>
+        <v>109737</v>
       </c>
       <c r="E39" t="n">
-        <v>21600</v>
+        <v>3703</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -2686,21 +2686,21 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>95044</v>
+        <v>109444</v>
       </c>
       <c r="D40" t="n">
-        <v>107044</v>
+        <v>123844</v>
       </c>
       <c r="E40" t="n">
-        <v>12000</v>
+        <v>14400</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>C4_3</t>
+          <t>C5_3</t>
         </is>
       </c>
       <c r="G40" t="n">
@@ -2713,21 +2713,21 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-1</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>95044</v>
+        <v>109737</v>
       </c>
       <c r="D41" t="n">
-        <v>109444</v>
+        <v>120537</v>
       </c>
       <c r="E41" t="n">
-        <v>14400</v>
+        <v>10800</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>C4_3</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="G41" t="n">
@@ -2744,17 +2744,17 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>109444</v>
+        <v>109737</v>
       </c>
       <c r="D42" t="n">
-        <v>123844</v>
+        <v>122697</v>
       </c>
       <c r="E42" t="n">
-        <v>14400</v>
+        <v>12960</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>C5_3</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="G42" t="n">
@@ -2818,25 +2818,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-1</t>
+          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_0</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="D2" t="n">
-        <v>4550</v>
+        <v>14600</v>
       </c>
       <c r="E2" t="n">
-        <v>4320</v>
+        <v>14400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -2845,25 +2845,25 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-2</t>
+          <t>Industrial Cleaning Machine2-2</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>230</v>
       </c>
       <c r="D3" t="n">
-        <v>10598</v>
+        <v>4550</v>
       </c>
       <c r="E3" t="n">
-        <v>10368</v>
+        <v>4320</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -2872,7 +2872,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>New_AUTOMATED_CONVEYING_ARM_1_9</t>
+          <t>Industrial Cleaning Machine1-1</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -2899,25 +2899,25 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>New_PRECISION_FILLING_MACHINE_2_0</t>
+          <t>Automated Conveying Arm1-1</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="D5" t="n">
-        <v>5650</v>
+        <v>10598</v>
       </c>
       <c r="E5" t="n">
-        <v>5400</v>
+        <v>10368</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -2926,17 +2926,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm2-1</t>
+          <t>Precision Filling Machine2-1</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>250</v>
       </c>
       <c r="D6" t="n">
-        <v>4570</v>
+        <v>5650</v>
       </c>
       <c r="E6" t="n">
-        <v>4320</v>
+        <v>5400</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -2953,25 +2953,25 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-4</t>
+          <t>New_AUTOMATED_CONVEYING_ARM_1_7</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>340</v>
+        <v>250</v>
       </c>
       <c r="D7" t="n">
-        <v>8980</v>
+        <v>4570</v>
       </c>
       <c r="E7" t="n">
-        <v>8640</v>
+        <v>4320</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -2980,21 +2980,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>Industrial Cleaning Machine2-4</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5650</v>
+        <v>340</v>
       </c>
       <c r="D8" t="n">
-        <v>23650</v>
+        <v>8980</v>
       </c>
       <c r="E8" t="n">
-        <v>18000</v>
+        <v>8640</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -3007,17 +3007,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-3</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>5650</v>
       </c>
       <c r="D9" t="n">
-        <v>12850</v>
+        <v>23650</v>
       </c>
       <c r="E9" t="n">
-        <v>7200</v>
+        <v>18000</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -3034,21 +3034,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-1</t>
+          <t>New_INDUSTRIAL_CLEANING_MACHINE_2_9</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>8980</v>
+        <v>5650</v>
       </c>
       <c r="D10" t="n">
-        <v>23380</v>
+        <v>12850</v>
       </c>
       <c r="E10" t="n">
-        <v>14400</v>
+        <v>7200</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -3061,17 +3061,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm1-3</t>
+          <t>Precision Filling Machine2-3</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>8980</v>
       </c>
       <c r="D11" t="n">
-        <v>18580</v>
+        <v>23380</v>
       </c>
       <c r="E11" t="n">
-        <v>9600</v>
+        <v>14400</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -3079,7 +3079,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -3088,25 +3088,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-4</t>
+          <t>New_AUTOMATED_CONVEYING_ARM_1_7</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9495</v>
+        <v>8980</v>
       </c>
       <c r="D12" t="n">
-        <v>23895</v>
+        <v>18580</v>
       </c>
       <c r="E12" t="n">
-        <v>14400</v>
+        <v>9600</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-4</t>
+          <t>Precision Filling Machine1-3</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -3133,7 +3133,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -3142,21 +3142,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-3</t>
+          <t>Precision Filling Machine2-5</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>11148</v>
+        <v>18004</v>
       </c>
       <c r="D14" t="n">
-        <v>38148</v>
+        <v>24484</v>
       </c>
       <c r="E14" t="n">
-        <v>27000</v>
+        <v>6480</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>C3_1</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -3169,25 +3169,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>New_AUTOMATED_CONVEYING_ARM_1_9</t>
+          <t>New_AUTOMATED_CONVEYING_ARM_2_8</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>11148</v>
+        <v>18004</v>
       </c>
       <c r="D15" t="n">
-        <v>29148</v>
+        <v>23188</v>
       </c>
       <c r="E15" t="n">
-        <v>18000</v>
+        <v>5184</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>C3_1</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -3196,25 +3196,25 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-5</t>
+          <t>Precision Filling Machine2-3</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>18004</v>
+        <v>23380</v>
       </c>
       <c r="D16" t="n">
-        <v>24484</v>
+        <v>28009</v>
       </c>
       <c r="E16" t="n">
-        <v>6480</v>
+        <v>4629</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -3223,25 +3223,25 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm2-2</t>
+          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_5</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>18004</v>
+        <v>23650</v>
       </c>
       <c r="D17" t="n">
-        <v>23188</v>
+        <v>41650</v>
       </c>
       <c r="E17" t="n">
-        <v>5184</v>
+        <v>18000</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>C3_1</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -3250,21 +3250,21 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-5</t>
+          <t>New_PRECISION_FILLING_MACHINE_2_0</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23380</v>
+        <v>23738</v>
       </c>
       <c r="D18" t="n">
-        <v>28009</v>
+        <v>50738</v>
       </c>
       <c r="E18" t="n">
-        <v>4629</v>
+        <v>27000</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -3277,21 +3277,21 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine2-1</t>
+          <t>New_AUTOMATED_CONVEYING_ARM_2_8</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>24484</v>
+        <v>23738</v>
       </c>
       <c r="D19" t="n">
-        <v>36484</v>
+        <v>41738</v>
       </c>
       <c r="E19" t="n">
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>C4_1</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -3304,17 +3304,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-3</t>
+          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_3</t>
         </is>
       </c>
       <c r="C20" t="n">
         <v>24484</v>
       </c>
       <c r="D20" t="n">
-        <v>38884</v>
+        <v>36484</v>
       </c>
       <c r="E20" t="n">
-        <v>14400</v>
+        <v>12000</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -3331,25 +3331,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-5</t>
+          <t>New_INDUSTRIAL_CLEANING_MACHINE_2_9</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>24909</v>
+        <v>24484</v>
       </c>
       <c r="D21" t="n">
-        <v>31081</v>
+        <v>38884</v>
       </c>
       <c r="E21" t="n">
-        <v>6172</v>
+        <v>14400</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>C4_1</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_4</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_2_4</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3412,21 +3412,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Precision Filling Machine1-5</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>38148</v>
+        <v>38884</v>
       </c>
       <c r="D24" t="n">
-        <v>41851</v>
+        <v>53284</v>
       </c>
       <c r="E24" t="n">
-        <v>3703</v>
+        <v>14400</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>C5_1</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -3439,21 +3439,21 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_4</t>
+          <t>Precision Filling Machine1-2</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>38884</v>
+        <v>50738</v>
       </c>
       <c r="D25" t="n">
-        <v>53284</v>
+        <v>54441</v>
       </c>
       <c r="E25" t="n">
-        <v>14400</v>
+        <v>3703</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>C5_1</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -3466,21 +3466,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Automatic Sensing Multi-Function Machine2-1</t>
+          <t>Precision Filling Machine2-5</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>46459</v>
+        <v>53284</v>
       </c>
       <c r="D26" t="n">
-        <v>64459</v>
+        <v>59764</v>
       </c>
       <c r="E26" t="n">
-        <v>18000</v>
+        <v>6480</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>C3_2</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -3493,17 +3493,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Precision Filling Machine2-5</t>
+          <t>New_AUTOMATED_CONVEYING_ARM_1_7</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>53284</v>
       </c>
       <c r="D27" t="n">
-        <v>59764</v>
+        <v>58468</v>
       </c>
       <c r="E27" t="n">
-        <v>6480</v>
+        <v>5184</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -3511,7 +3511,7 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -3520,21 +3520,21 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>New_AUTOMATED_CONVEYING_ARM_1_9</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>53284</v>
+        <v>59764</v>
       </c>
       <c r="D28" t="n">
-        <v>58468</v>
+        <v>71764</v>
       </c>
       <c r="E28" t="n">
-        <v>5184</v>
+        <v>12000</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C3_2</t>
+          <t>C4_2</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -3547,17 +3547,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_2</t>
+          <t>New_INDUSTRIAL_CLEANING_MACHINE_2_9</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>59764</v>
       </c>
       <c r="D29" t="n">
-        <v>71764</v>
+        <v>74164</v>
       </c>
       <c r="E29" t="n">
-        <v>12000</v>
+        <v>14400</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -3574,25 +3574,25 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-4</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>59764</v>
+        <v>73009</v>
       </c>
       <c r="D30" t="n">
-        <v>74164</v>
+        <v>91009</v>
       </c>
       <c r="E30" t="n">
-        <v>14400</v>
+        <v>18000</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C4_2</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -3601,21 +3601,21 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_2</t>
+          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_2_4</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>72314</v>
+        <v>74164</v>
       </c>
       <c r="D31" t="n">
-        <v>83114</v>
+        <v>88564</v>
       </c>
       <c r="E31" t="n">
-        <v>10800</v>
+        <v>14400</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>C5_2</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -3628,25 +3628,25 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_1</t>
+          <t>New_PRECISION_FILLING_MACHINE_2_0</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>72314</v>
+        <v>88564</v>
       </c>
       <c r="D32" t="n">
-        <v>85274</v>
+        <v>95044</v>
       </c>
       <c r="E32" t="n">
-        <v>12960</v>
+        <v>6480</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>C3_3</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -3655,21 +3655,21 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_5</t>
+          <t>New_AUTOMATED_CONVEYING_ARM_1_7</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>73009</v>
+        <v>88564</v>
       </c>
       <c r="D33" t="n">
-        <v>91009</v>
+        <v>93748</v>
       </c>
       <c r="E33" t="n">
-        <v>18000</v>
+        <v>5184</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>C3_3</t>
         </is>
       </c>
       <c r="G33" t="n">
@@ -3682,21 +3682,21 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_4</t>
+          <t>High-speed Polishing Machine1-1</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>74164</v>
+        <v>91009</v>
       </c>
       <c r="D34" t="n">
-        <v>88564</v>
+        <v>116209</v>
       </c>
       <c r="E34" t="n">
-        <v>14400</v>
+        <v>25200</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C5_2</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -3709,21 +3709,21 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>New_PRECISION_FILLING_MACHINE_2_0</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>88564</v>
+        <v>95044</v>
       </c>
       <c r="D35" t="n">
-        <v>95044</v>
+        <v>107044</v>
       </c>
       <c r="E35" t="n">
-        <v>6480</v>
+        <v>12000</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C3_3</t>
+          <t>C4_3</t>
         </is>
       </c>
       <c r="G35" t="n">
@@ -3736,21 +3736,21 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Automated Conveying Arm2-4</t>
+          <t>Industrial Cleaning Machine2-1</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>88564</v>
+        <v>95044</v>
       </c>
       <c r="D36" t="n">
-        <v>93748</v>
+        <v>109444</v>
       </c>
       <c r="E36" t="n">
-        <v>5184</v>
+        <v>14400</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C3_3</t>
+          <t>C4_3</t>
         </is>
       </c>
       <c r="G36" t="n">
@@ -3763,25 +3763,25 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>New_AUTOMATIC_SENSING_MULTI_FUNCTION_MACHINE_1_4</t>
+          <t>New_PRECISION_FILLING_MACHINE_2_0</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>88989</v>
+        <v>95469</v>
       </c>
       <c r="D37" t="n">
-        <v>96189</v>
+        <v>101641</v>
       </c>
       <c r="E37" t="n">
-        <v>7200</v>
+        <v>6172</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -3790,17 +3790,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine1-5</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>88989</v>
+        <v>101641</v>
       </c>
       <c r="D38" t="n">
-        <v>110589</v>
+        <v>108841</v>
       </c>
       <c r="E38" t="n">
-        <v>21600</v>
+        <v>7200</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -3817,25 +3817,25 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>New_HIGH_SPEED_POLISHING_MACHINE_2_2</t>
+          <t>New_INDUSTRIAL_CLEANING_MACHINE_1_9</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>91009</v>
+        <v>101641</v>
       </c>
       <c r="D39" t="n">
-        <v>116209</v>
+        <v>123241</v>
       </c>
       <c r="E39" t="n">
-        <v>25200</v>
+        <v>21600</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -3844,25 +3844,25 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>High-speed Polishing Machine1-1</t>
+          <t>High-speed Polishing Machine2-1</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>95044</v>
+        <v>109201</v>
       </c>
       <c r="D40" t="n">
-        <v>107044</v>
+        <v>120001</v>
       </c>
       <c r="E40" t="n">
-        <v>12000</v>
+        <v>10800</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>C4_3</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -3871,25 +3871,25 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Industrial Cleaning Machine2-3</t>
+          <t>Automatic Sensing Multi-Function Machine1-1</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>95044</v>
+        <v>109201</v>
       </c>
       <c r="D41" t="n">
-        <v>109444</v>
+        <v>122161</v>
       </c>
       <c r="E41" t="n">
-        <v>14400</v>
+        <v>12960</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>C4_3</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -3960,7 +3960,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -3970,10 +3970,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -3996,10 +3996,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -4012,7 +4012,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>采购费用475000/500000</t>
+          <t>采购费用490000/500000</t>
         </is>
       </c>
     </row>

</xml_diff>